<commit_message>
Mubasshera Rizvi Update 03_Test_Cases
</commit_message>
<xml_diff>
--- a/03_Test_Cases/Test_Cases.xlsx
+++ b/03_Test_Cases/Test_Cases.xlsx
@@ -1,29 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
-  <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\AutomationExercise_Automation_Project_Templates\03_Test_Cases\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD6C12FD-F0EB-4B1B-8559-5C13AC53D99A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="7" rupBuild="4505"/>
+  <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="19416" windowHeight="10296" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="Login" sheetId="1" r:id="rId1"/>
     <sheet name="Registration" sheetId="2" r:id="rId2"/>
     <sheet name="Cart" sheetId="3" r:id="rId3"/>
     <sheet name="Checkout" sheetId="4" r:id="rId4"/>
+    <sheet name="Navigatoion" sheetId="5" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="116">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -281,13 +276,103 @@
   </si>
   <si>
     <t>Checkout cancelled</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>TC021</t>
+  </si>
+  <si>
+    <t>TC022</t>
+  </si>
+  <si>
+    <t>TC023</t>
+  </si>
+  <si>
+    <t>TC024</t>
+  </si>
+  <si>
+    <t>TC025</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Verify Products Page Navigation</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Click Products menu</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Verify Cart Page Navigation</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Verify Login Page Navigation</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Verify Category Navigation</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Verify Add to Cart Flow</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Click Cart menu</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Click Signup/Login menu</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Click Women → Dress category</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Add product → Open cart</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Navigation</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> User navigates to Products page</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> User navigates to Cart page</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> User navigates to Login page</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Women products should display</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Product visible in cart</t>
+  </si>
+  <si>
+    <t>Navigated to products page</t>
+  </si>
+  <si>
+    <t>Navigated to cart page</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Navigated to login page</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Category element not found</t>
+  </si>
+  <si>
+    <t>Executed</t>
+  </si>
+  <si>
+    <t>Result</t>
+  </si>
+  <si>
+    <t>Pass</t>
+  </si>
+  <si>
+    <t>Fail</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -619,18 +704,18 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G6"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="36.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="25.54296875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="36.21875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="25.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -653,7 +738,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -673,7 +758,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7">
       <c r="A3" t="s">
         <v>13</v>
       </c>
@@ -693,7 +778,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7">
       <c r="A4" t="s">
         <v>17</v>
       </c>
@@ -713,7 +798,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7">
       <c r="A5" t="s">
         <v>20</v>
       </c>
@@ -733,7 +818,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7">
       <c r="A6" t="s">
         <v>24</v>
       </c>
@@ -759,20 +844,20 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G6"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="10.90625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.36328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.7265625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="28.08984375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="25.54296875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.77734375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="28.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="25.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -795,7 +880,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7">
       <c r="A2" t="s">
         <v>28</v>
       </c>
@@ -815,7 +900,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7">
       <c r="A3" t="s">
         <v>33</v>
       </c>
@@ -835,7 +920,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7">
       <c r="A4" t="s">
         <v>36</v>
       </c>
@@ -855,7 +940,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7">
       <c r="A5" t="s">
         <v>39</v>
       </c>
@@ -875,7 +960,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7">
       <c r="A6" t="s">
         <v>42</v>
       </c>
@@ -901,20 +986,20 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G6"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="10.90625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.88671875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="23" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.26953125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="24.453125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="28.90625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.21875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="24.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="28.88671875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -937,7 +1022,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7">
       <c r="A2" t="s">
         <v>46</v>
       </c>
@@ -957,7 +1042,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7">
       <c r="A3" t="s">
         <v>51</v>
       </c>
@@ -977,7 +1062,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7">
       <c r="A4" t="s">
         <v>55</v>
       </c>
@@ -997,7 +1082,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7">
       <c r="A5" t="s">
         <v>59</v>
       </c>
@@ -1017,7 +1102,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7">
       <c r="A6" t="s">
         <v>63</v>
       </c>
@@ -1043,20 +1128,20 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:G6"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:J23"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="10.90625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.26953125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.54296875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="26.26953125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="21.36328125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.54296875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11" customWidth="1"/>
+    <col min="2" max="2" width="22.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="26.21875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="21.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1079,7 +1164,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7">
       <c r="A2" t="s">
         <v>66</v>
       </c>
@@ -1099,7 +1184,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7">
       <c r="A3" t="s">
         <v>71</v>
       </c>
@@ -1119,7 +1204,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7">
       <c r="A4" t="s">
         <v>74</v>
       </c>
@@ -1139,7 +1224,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7">
       <c r="A5" t="s">
         <v>78</v>
       </c>
@@ -1159,7 +1244,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7">
       <c r="A6" t="s">
         <v>82</v>
       </c>
@@ -1177,9 +1262,209 @@
       </c>
       <c r="G6" t="s">
         <v>12</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7">
+      <c r="B10" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="23" spans="10:10">
+      <c r="J23" t="s">
+        <v>86</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:J12"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="11" customWidth="1"/>
+    <col min="2" max="2" width="27.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.6640625" customWidth="1"/>
+    <col min="4" max="4" width="28" customWidth="1"/>
+    <col min="5" max="5" width="28.6640625" customWidth="1"/>
+    <col min="6" max="6" width="25.21875" customWidth="1"/>
+    <col min="7" max="7" width="11.77734375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10">
+      <c r="A2" t="s">
+        <v>87</v>
+      </c>
+      <c r="B2" t="s">
+        <v>92</v>
+      </c>
+      <c r="C2" t="s">
+        <v>102</v>
+      </c>
+      <c r="D2" t="s">
+        <v>93</v>
+      </c>
+      <c r="E2" t="s">
+        <v>103</v>
+      </c>
+      <c r="F2" t="s">
+        <v>108</v>
+      </c>
+      <c r="G2" t="s">
+        <v>112</v>
+      </c>
+      <c r="H2" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10">
+      <c r="A3" t="s">
+        <v>88</v>
+      </c>
+      <c r="B3" t="s">
+        <v>94</v>
+      </c>
+      <c r="C3" t="s">
+        <v>102</v>
+      </c>
+      <c r="D3" t="s">
+        <v>98</v>
+      </c>
+      <c r="E3" t="s">
+        <v>104</v>
+      </c>
+      <c r="F3" t="s">
+        <v>109</v>
+      </c>
+      <c r="G3" t="s">
+        <v>112</v>
+      </c>
+      <c r="H3" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10">
+      <c r="A4" t="s">
+        <v>89</v>
+      </c>
+      <c r="B4" t="s">
+        <v>95</v>
+      </c>
+      <c r="C4" t="s">
+        <v>102</v>
+      </c>
+      <c r="D4" t="s">
+        <v>99</v>
+      </c>
+      <c r="E4" t="s">
+        <v>105</v>
+      </c>
+      <c r="F4" t="s">
+        <v>110</v>
+      </c>
+      <c r="G4" t="s">
+        <v>112</v>
+      </c>
+      <c r="H4" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10">
+      <c r="A5" t="s">
+        <v>90</v>
+      </c>
+      <c r="B5" t="s">
+        <v>96</v>
+      </c>
+      <c r="C5" t="s">
+        <v>102</v>
+      </c>
+      <c r="D5" t="s">
+        <v>100</v>
+      </c>
+      <c r="E5" t="s">
+        <v>106</v>
+      </c>
+      <c r="F5" t="s">
+        <v>111</v>
+      </c>
+      <c r="G5" t="s">
+        <v>12</v>
+      </c>
+      <c r="H5" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10">
+      <c r="A6" t="s">
+        <v>91</v>
+      </c>
+      <c r="B6" t="s">
+        <v>97</v>
+      </c>
+      <c r="C6" t="s">
+        <v>102</v>
+      </c>
+      <c r="D6" t="s">
+        <v>101</v>
+      </c>
+      <c r="E6" t="s">
+        <v>107</v>
+      </c>
+      <c r="F6" t="s">
+        <v>107</v>
+      </c>
+      <c r="G6" t="s">
+        <v>112</v>
+      </c>
+      <c r="H6" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10">
+      <c r="C8" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10">
+      <c r="B10" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10">
+      <c r="J12" t="s">
+        <v>86</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
[Mubasshera Rizvi] Add Navigation Test
</commit_message>
<xml_diff>
--- a/03_Test_Cases/Test_Cases.xlsx
+++ b/03_Test_Cases/Test_Cases.xlsx
@@ -365,7 +365,7 @@
     <t>Pass</t>
   </si>
   <si>
-    <t>Fail</t>
+    <t xml:space="preserve"> Pass </t>
   </si>
 </sst>
 </file>
@@ -1420,7 +1420,7 @@
         <v>12</v>
       </c>
       <c r="H5" t="s">
-        <v>115</v>
+        <v>86</v>
       </c>
     </row>
     <row r="6" spans="1:10">
@@ -1446,7 +1446,7 @@
         <v>112</v>
       </c>
       <c r="H6" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="8" spans="1:10">

</xml_diff>

<commit_message>
[Mubasshera Rizvi] Updated Test_cases File
</commit_message>
<xml_diff>
--- a/03_Test_Cases/Test_Cases.xlsx
+++ b/03_Test_Cases/Test_Cases.xlsx
@@ -1417,10 +1417,10 @@
         <v>111</v>
       </c>
       <c r="G5" t="s">
-        <v>12</v>
+        <v>112</v>
       </c>
       <c r="H5" t="s">
-        <v>86</v>
+        <v>114</v>
       </c>
     </row>
     <row r="6" spans="1:10">

</xml_diff>